<commit_message>
Add file-naming rule check; sharpen sample occupancy item
- New 'File naming' rule: reads a pattern like Client_Q3-2026_<Document> from the checklist item and checks every file name against it, without the model
- Sample checklist: occupancy item now points at the deck's portfolio slide

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JoZ643NDKMrfQxG5cBYjE8
</commit_message>
<xml_diff>
--- a/tickmark-sample-files/Investor_Pack_QA_Checklist.xlsx
+++ b/tickmark-sample-files/Investor_Pack_QA_Checklist.xlsx
@@ -445,6 +445,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -491,7 +492,6 @@
           <t>AM</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -512,7 +512,6 @@
           <t>AM</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -533,7 +532,6 @@
           <t>AM</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -554,7 +552,6 @@
           <t>AM</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -575,7 +572,6 @@
           <t>AM</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -596,7 +592,6 @@
           <t>AM</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -617,7 +612,6 @@
           <t>AM</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -638,7 +632,6 @@
           <t>AM</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -659,7 +652,6 @@
           <t>AM</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -680,7 +672,6 @@
           <t>AM</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -701,7 +692,6 @@
           <t>AM</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -714,7 +704,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Each property section states its occupancy rate.</t>
+          <t>Each property on the deck's portfolio slide states its occupancy rate.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -722,7 +712,6 @@
           <t>AM</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -743,7 +732,6 @@
           <t>AM</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -764,7 +752,6 @@
           <t>AM</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -785,7 +772,6 @@
           <t>AM</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -806,7 +792,6 @@
           <t>AM</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>